<commit_message>
feat: add Genba MNG export template file
</commit_message>
<xml_diff>
--- a/public/tamplate-xlsx/Genba_MNG_Export_Tamplate.xlsx
+++ b/public/tamplate-xlsx/Genba_MNG_Export_Tamplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ict\www-wsl\qms\public\tamplate-xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3ABD19-C5BC-4314-861B-A2C196F25578}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B0EB970-C803-4DC9-92BC-6CFE7654A848}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{B477D971-9BD2-431E-A60E-0A4EA9480CFF}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>Departement</t>
   </si>
@@ -88,13 +88,40 @@
   </si>
   <si>
     <t>Robot no. 2 Parameter welding time utk 3 item berbeda dengan standard. SOP dan Check sheet berbeda dengan Aktual. Contoh : part Leg Sub Assy W2 standard 25 cycle, Aktual 35 cycle</t>
+  </si>
+  <si>
+    <t>Nomor Dokumen</t>
+  </si>
+  <si>
+    <t>Tanggal Terbit</t>
+  </si>
+  <si>
+    <t>No Revisi</t>
+  </si>
+  <si>
+    <t>Halaman</t>
+  </si>
+  <si>
+    <t>FO-08-09</t>
+  </si>
+  <si>
+    <t>Manajemen</t>
+  </si>
+  <si>
+    <t>(Tanggal di Export)</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>1 dari 1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +172,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -382,7 +415,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -423,7 +456,69 @@
     <xf numFmtId="15" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="15" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="6" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="4" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -436,70 +531,15 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="6" fillId="3" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="4" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -874,8 +914,8 @@
     <col min="7" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="19.7109375" customWidth="1"/>
     <col min="9" max="9" width="45.42578125" customWidth="1"/>
-    <col min="10" max="10" width="16.85546875" customWidth="1"/>
-    <col min="11" max="11" width="18.42578125" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.28515625" customWidth="1"/>
     <col min="14" max="14" width="21.28515625" customWidth="1"/>
     <col min="15" max="15" width="13.42578125" customWidth="1"/>
@@ -885,68 +925,88 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="15.75" customHeight="1">
-      <c r="B2" s="15"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="19" t="s">
+      <c r="B2" s="35"/>
+      <c r="C2" s="36"/>
+      <c r="D2" s="36"/>
+      <c r="E2" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="37"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="40"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="39" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="3" spans="2:11" ht="15" customHeight="1">
-      <c r="B3" s="17"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="38"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="40"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="28"/>
+      <c r="J3" s="39" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" s="39" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="4" spans="2:11" ht="15.75" customHeight="1">
-      <c r="B4" s="17"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="38"/>
-      <c r="J4" s="14"/>
-      <c r="K4" s="40"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="27"/>
+      <c r="H4" s="27"/>
+      <c r="I4" s="28"/>
+      <c r="J4" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" s="39" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="5" spans="2:11" ht="15.75" customHeight="1">
-      <c r="B5" s="17"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="38"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="40"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="40" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="6" spans="2:11" ht="15" customHeight="1">
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="39"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="40"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="41" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="7" spans="2:11">
       <c r="B7" s="1"/>
@@ -966,51 +1026,51 @@
       <c r="H7" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="25" t="s">
+      <c r="I7" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
+      <c r="J7" s="32"/>
+      <c r="K7" s="32"/>
     </row>
     <row r="8" spans="2:11">
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="G8" s="26" t="s">
+      <c r="G8" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="H8" s="26" t="s">
+      <c r="H8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="26" t="s">
+      <c r="I8" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="26"/>
-      <c r="K8" s="26"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="21"/>
     </row>
     <row r="9" spans="2:11">
-      <c r="B9" s="31"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="26"/>
-      <c r="K9" s="26"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
     </row>
     <row r="10" spans="2:11">
       <c r="B10" s="3"/>
@@ -1020,9 +1080,9 @@
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="12"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="27"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="33"/>
     </row>
     <row r="11" spans="2:11" ht="60" customHeight="1">
       <c r="B11" s="5">
@@ -1046,31 +1106,34 @@
       <c r="H11" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I11" s="28" t="s">
+      <c r="I11" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="J11" s="28"/>
-      <c r="K11" s="28"/>
+      <c r="J11" s="34"/>
+      <c r="K11" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="B2:D5"/>
     <mergeCell ref="F8:F9"/>
     <mergeCell ref="G8:G9"/>
     <mergeCell ref="H8:H9"/>
     <mergeCell ref="E2:I6"/>
     <mergeCell ref="I7:K7"/>
     <mergeCell ref="I8:K9"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="B2:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="K5" numberStoredAsText="1"/>
+  </ignoredErrors>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>